<commit_message>
reduced latency. bettery styles. save points during stepping with step name. plot them.
</commit_message>
<xml_diff>
--- a/sensor_app/example_config.xlsx
+++ b/sensor_app/example_config.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Instruments" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Channels" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Control Loops" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Interlocks" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Logging" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Settings" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Step Series" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instruments" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Channels" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control Loops" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interlocks" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Logging" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Step Series" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2274,7 +2274,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2292,20 +2292,25 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
           <t>SP: reactor_temp (degC)</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>dummy_output_slider</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>dummy_output_selector</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>Hold Time (s)</t>
         </is>
@@ -2317,27 +2322,32 @@
           <t>Tolerance</t>
         </is>
       </c>
-      <c r="B3" t="n">
-        <v>5</v>
-      </c>
       <c r="C3" t="n">
         <v>5</v>
       </c>
+      <c r="D3" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
         <v>1</v>
       </c>
-      <c r="B4" t="n">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
         <v>50</v>
       </c>
-      <c r="C4" t="n">
+      <c r="D4" t="n">
         <v>25</v>
       </c>
-      <c r="D4" t="n">
-        <v>0</v>
-      </c>
       <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
         <v>5</v>
       </c>
     </row>
@@ -2345,16 +2355,21 @@
       <c r="A5" t="n">
         <v>2</v>
       </c>
-      <c r="B5" t="n">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
         <v>75</v>
       </c>
-      <c r="C5" t="n">
+      <c r="D5" t="n">
         <v>50</v>
       </c>
-      <c r="D5" t="n">
-        <v>1</v>
-      </c>
       <c r="E5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" t="n">
         <v>5</v>
       </c>
     </row>
@@ -2362,16 +2377,21 @@
       <c r="A6" t="n">
         <v>3</v>
       </c>
-      <c r="B6" t="n">
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
         <v>100</v>
       </c>
-      <c r="C6" t="n">
+      <c r="D6" t="n">
         <v>75</v>
       </c>
-      <c r="D6" t="n">
+      <c r="E6" t="n">
         <v>2</v>
       </c>
-      <c r="E6" t="n">
+      <c r="F6" t="n">
         <v>5</v>
       </c>
     </row>

</xml_diff>

<commit_message>
added test sequence selector
</commit_message>
<xml_diff>
--- a/sensor_app/example_config.xlsx
+++ b/sensor_app/example_config.xlsx
@@ -2318,7 +2318,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2336,35 +2336,40 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>Test Sequence</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>SP: reactor_temp (degC)</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>dummy_out_slider</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>dummy_out_selector</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>Watch: dummy_out_slider</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>Watch: temperature (C)</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>Hold Time (s)</t>
         </is>
@@ -2376,16 +2381,16 @@
           <t>Tolerance</t>
         </is>
       </c>
-      <c r="C3" t="n">
-        <v>5</v>
-      </c>
       <c r="D3" t="n">
         <v>5</v>
       </c>
-      <c r="F3" t="n">
+      <c r="E3" t="n">
         <v>5</v>
       </c>
       <c r="G3" t="n">
+        <v>5</v>
+      </c>
+      <c r="H3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -2395,25 +2400,30 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
+          <t>Ramp Up</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="C4" t="n">
+      <c r="D4" t="n">
         <v>50</v>
       </c>
-      <c r="D4" t="n">
+      <c r="E4" t="n">
         <v>25</v>
       </c>
-      <c r="E4" t="n">
-        <v>0</v>
-      </c>
       <c r="F4" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="G4" t="n">
         <v>50</v>
       </c>
       <c r="H4" t="n">
+        <v>50</v>
+      </c>
+      <c r="I4" t="n">
         <v>5</v>
       </c>
     </row>
@@ -2423,25 +2433,30 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
+          <t>Ramp Up</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="C5" t="n">
+      <c r="D5" t="n">
         <v>75</v>
       </c>
-      <c r="D5" t="n">
+      <c r="E5" t="n">
         <v>50</v>
       </c>
-      <c r="E5" t="n">
-        <v>1</v>
-      </c>
       <c r="F5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" t="n">
         <v>10</v>
       </c>
-      <c r="G5" t="n">
+      <c r="H5" t="n">
         <v>50</v>
       </c>
-      <c r="H5" t="n">
+      <c r="I5" t="n">
         <v>5</v>
       </c>
     </row>
@@ -2451,25 +2466,129 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
+          <t>Ramp Up</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
           <t>High</t>
         </is>
       </c>
-      <c r="C6" t="n">
+      <c r="D6" t="n">
         <v>100</v>
       </c>
-      <c r="D6" t="n">
+      <c r="E6" t="n">
         <v>75</v>
       </c>
-      <c r="E6" t="n">
+      <c r="F6" t="n">
         <v>2</v>
       </c>
-      <c r="F6" t="n">
+      <c r="G6" t="n">
         <v>20</v>
       </c>
-      <c r="G6" t="n">
+      <c r="H6" t="n">
         <v>50</v>
       </c>
-      <c r="H6" t="n">
+      <c r="I6" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Thermal Cycle</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>100</v>
+      </c>
+      <c r="E7" t="n">
+        <v>75</v>
+      </c>
+      <c r="F7" t="n">
+        <v>2</v>
+      </c>
+      <c r="G7" t="n">
+        <v>75</v>
+      </c>
+      <c r="H7" t="n">
+        <v>100</v>
+      </c>
+      <c r="I7" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>2</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Thermal Cycle</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Cold</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>30</v>
+      </c>
+      <c r="E8" t="n">
+        <v>10</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" t="n">
+        <v>10</v>
+      </c>
+      <c r="H8" t="n">
+        <v>30</v>
+      </c>
+      <c r="I8" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>3</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Thermal Cycle</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>100</v>
+      </c>
+      <c r="E9" t="n">
+        <v>75</v>
+      </c>
+      <c r="F9" t="n">
+        <v>2</v>
+      </c>
+      <c r="G9" t="n">
+        <v>75</v>
+      </c>
+      <c r="H9" t="n">
+        <v>100</v>
+      </c>
+      <c r="I9" t="n">
         <v>5</v>
       </c>
     </row>

</xml_diff>